<commit_message>
Round 1 revision: neutral styling, unified task/answer formats, add missing sheets, rubric rebalance plan
</commit_message>
<xml_diff>
--- a/股票组合风险分析_任务文件.xlsx
+++ b/股票组合风险分析_任务文件.xlsx
@@ -10,8 +10,11 @@
     <sheet name="原始行情" sheetId="1" r:id="rId1"/>
     <sheet name="参数设置" sheetId="2" r:id="rId2"/>
     <sheet name="组合分析" sheetId="3" r:id="rId3"/>
-    <sheet name="压力测试" sheetId="4" r:id="rId4"/>
-    <sheet name="投资仪表盘" sheetId="5" r:id="rId5"/>
+    <sheet name="月度收益" sheetId="4" r:id="rId4"/>
+    <sheet name="压力测试" sheetId="5" r:id="rId5"/>
+    <sheet name="投资仪表盘" sheetId="6" r:id="rId6"/>
+    <sheet name="行业风险归因" sheetId="7" r:id="rId7"/>
+    <sheet name="风险回测" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">原始行情!$A$2:$G$290</definedName>
@@ -21,9 +24,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1114" uniqueCount="98">
-  <si>
-    <t>模拟股票月度行情（数据已完整提供，无需外部检索）</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1186" uniqueCount="132">
+  <si>
+    <t>模拟股票月度行情</t>
   </si>
   <si>
     <t>日期</t>
@@ -206,10 +209,7 @@
     <t>增长反弹</t>
   </si>
   <si>
-    <t>股票组合收益与风险分析</t>
-  </si>
-  <si>
-    <t>蓝色单元格为公式结果；所有收益率、风险指标与贡献值均应保持公式联动。</t>
+    <t>股票组合分析</t>
   </si>
   <si>
     <t>最新价</t>
@@ -245,7 +245,7 @@
     <t>加权Beta贡献</t>
   </si>
   <si>
-    <t>月度VaR贡献</t>
+    <t>95%单尾月度VaR贡献</t>
   </si>
   <si>
     <t>配置判断</t>
@@ -278,10 +278,25 @@
     <t>基准年化收益率</t>
   </si>
   <si>
-    <t>股票组合情景压力测试</t>
-  </si>
-  <si>
-    <t>按行业冲击映射至每只股票，计算持仓市值和情景损益；负值代表亏损。</t>
+    <t>月份</t>
+  </si>
+  <si>
+    <t>基准月收益率</t>
+  </si>
+  <si>
+    <t>组合月收益率</t>
+  </si>
+  <si>
+    <t>组合累计净值</t>
+  </si>
+  <si>
+    <t>基准累计净值</t>
+  </si>
+  <si>
+    <t>组合回撤</t>
+  </si>
+  <si>
+    <t>压力测试</t>
   </si>
   <si>
     <t>情景</t>
@@ -305,16 +320,106 @@
     <t>风险判断</t>
   </si>
   <si>
-    <t>股票组合投资仪表盘</t>
+    <t>投资仪表盘</t>
   </si>
   <si>
     <t>95%单月VaR率</t>
   </si>
   <si>
-    <t>风险贡献最高的 5 只股票</t>
+    <t>VaR贡献前五持仓</t>
   </si>
   <si>
     <t>排名</t>
+  </si>
+  <si>
+    <t>行业风险归因</t>
+  </si>
+  <si>
+    <t>月末</t>
+  </si>
+  <si>
+    <t>加权组合收益</t>
+  </si>
+  <si>
+    <t>行业目标权重</t>
+  </si>
+  <si>
+    <t>样本协方差</t>
+  </si>
+  <si>
+    <t>Σw</t>
+  </si>
+  <si>
+    <t>VaR贡献</t>
+  </si>
+  <si>
+    <t>边际VaR</t>
+  </si>
+  <si>
+    <t>独立VaR</t>
+  </si>
+  <si>
+    <t>组合月方差</t>
+  </si>
+  <si>
+    <t>协方差组合VaR</t>
+  </si>
+  <si>
+    <t>贡献合计</t>
+  </si>
+  <si>
+    <t>分散化收益</t>
+  </si>
+  <si>
+    <t>最大风险贡献行业</t>
+  </si>
+  <si>
+    <t>风险回测</t>
+  </si>
+  <si>
+    <t>检验月末</t>
+  </si>
+  <si>
+    <t>实际组合月收益</t>
+  </si>
+  <si>
+    <t>前12月年化波动</t>
+  </si>
+  <si>
+    <t>前12月Beta</t>
+  </si>
+  <si>
+    <t>前12月跟踪误差</t>
+  </si>
+  <si>
+    <t>90%历史VaR率</t>
+  </si>
+  <si>
+    <t>90%历史ES率</t>
+  </si>
+  <si>
+    <t>VaR突破</t>
+  </si>
+  <si>
+    <t>前12月信息比率</t>
+  </si>
+  <si>
+    <t>实际损失率</t>
+  </si>
+  <si>
+    <t>主动月收益</t>
+  </si>
+  <si>
+    <t>突破次数</t>
+  </si>
+  <si>
+    <t>突破率</t>
+  </si>
+  <si>
+    <t>理论突破次数</t>
+  </si>
+  <si>
+    <t>回测状态</t>
   </si>
 </sst>
 </file>
@@ -327,7 +432,7 @@
     <numFmt numFmtId="166" formatCode="¥#,##0;[Red]-¥#,##0"/>
     <numFmt numFmtId="167" formatCode="0.00%;[Red]-0.00%"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -337,8 +442,8 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+      <color rgb="FF1F1F1F"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -346,36 +451,28 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF666666"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF7F6000"/>
+      <sz val="12"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -384,43 +481,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
+        <fgColor rgb="FFE7E6E6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4472C4"/>
+        <fgColor rgb="FFEDEDED"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2F75B5"/>
+        <fgColor rgb="FFF5F5F5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2F0D9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEAF2F8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF5B9BD5"/>
+        <fgColor rgb="FFFFF7E6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -452,12 +531,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -470,25 +547,41 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8696B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
@@ -783,9 +876,10 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="11.7109375" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" customWidth="1"/>
-    <col min="5" max="7" width="15.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="9.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="7" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -799,7 +893,7 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" ht="26" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -7461,8 +7555,8 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" customWidth="1"/>
-    <col min="3" max="3" width="38.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="3" max="3" width="40.7109375" customWidth="1"/>
     <col min="4" max="7" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7475,7 +7569,7 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" ht="26" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>39</v>
       </c>
@@ -7781,14 +7875,22 @@
   <dimension ref="A1:Q28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" customWidth="1"/>
-    <col min="4" max="16" width="14.7109375" customWidth="1"/>
-    <col min="17" max="17" width="13.7109375" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" customWidth="1"/>
+    <col min="4" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="8.7109375" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" customWidth="1"/>
+    <col min="12" max="12" width="20.7109375" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" customWidth="1"/>
+    <col min="14" max="15" width="13.7109375" customWidth="1"/>
+    <col min="16" max="16" width="16.7109375" customWidth="1"/>
+    <col min="17" max="17" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="26" customHeight="1">
+    <row r="1" spans="1:17" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>61</v>
       </c>
@@ -7809,28 +7911,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="1:17">
-      <c r="A2" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-    </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:17" ht="46" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -7841,46 +7922,46 @@
         <v>4</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="L5" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="M5" s="2" t="s">
         <v>55</v>
       </c>
       <c r="N5" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="O5" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="O5" s="2" t="s">
+      <c r="P5" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="P5" s="2" t="s">
+      <c r="Q5" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="Q5" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -7893,19 +7974,19 @@
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="12"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="12"/>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" spans="1:17">
@@ -7918,19 +7999,19 @@
       <c r="C7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="13"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="12"/>
+      <c r="M7" s="12"/>
+      <c r="N7" s="12"/>
+      <c r="O7" s="12"/>
+      <c r="P7" s="12"/>
       <c r="Q7" s="13"/>
     </row>
     <row r="8" spans="1:17">
@@ -7943,19 +8024,19 @@
       <c r="C8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
-      <c r="J8" s="13"/>
-      <c r="K8" s="13"/>
-      <c r="L8" s="13"/>
-      <c r="M8" s="13"/>
-      <c r="N8" s="13"/>
-      <c r="O8" s="13"/>
-      <c r="P8" s="13"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="12"/>
+      <c r="M8" s="12"/>
+      <c r="N8" s="12"/>
+      <c r="O8" s="12"/>
+      <c r="P8" s="12"/>
       <c r="Q8" s="13"/>
     </row>
     <row r="9" spans="1:17">
@@ -7968,19 +8049,19 @@
       <c r="C9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="13"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="13"/>
-      <c r="N9" s="13"/>
-      <c r="O9" s="13"/>
-      <c r="P9" s="13"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="12"/>
       <c r="Q9" s="13"/>
     </row>
     <row r="10" spans="1:17">
@@ -7993,19 +8074,19 @@
       <c r="C10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="13"/>
-      <c r="L10" s="13"/>
-      <c r="M10" s="13"/>
-      <c r="N10" s="13"/>
-      <c r="O10" s="13"/>
-      <c r="P10" s="13"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="12"/>
+      <c r="M10" s="12"/>
+      <c r="N10" s="12"/>
+      <c r="O10" s="12"/>
+      <c r="P10" s="12"/>
       <c r="Q10" s="13"/>
     </row>
     <row r="11" spans="1:17">
@@ -8018,19 +8099,19 @@
       <c r="C11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="13"/>
-      <c r="L11" s="13"/>
-      <c r="M11" s="13"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="13"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="12"/>
       <c r="Q11" s="13"/>
     </row>
     <row r="12" spans="1:17">
@@ -8043,19 +8124,19 @@
       <c r="C12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="13"/>
-      <c r="L12" s="13"/>
-      <c r="M12" s="13"/>
-      <c r="N12" s="13"/>
-      <c r="O12" s="13"/>
-      <c r="P12" s="13"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="12"/>
+      <c r="M12" s="12"/>
+      <c r="N12" s="12"/>
+      <c r="O12" s="12"/>
+      <c r="P12" s="12"/>
       <c r="Q12" s="13"/>
     </row>
     <row r="13" spans="1:17">
@@ -8068,19 +8149,19 @@
       <c r="C13" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
-      <c r="J13" s="13"/>
-      <c r="K13" s="13"/>
-      <c r="L13" s="13"/>
-      <c r="M13" s="13"/>
-      <c r="N13" s="13"/>
-      <c r="O13" s="13"/>
-      <c r="P13" s="13"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="12"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="12"/>
       <c r="Q13" s="13"/>
     </row>
     <row r="14" spans="1:17">
@@ -8093,19 +8174,19 @@
       <c r="C14" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13"/>
-      <c r="J14" s="13"/>
-      <c r="K14" s="13"/>
-      <c r="L14" s="13"/>
-      <c r="M14" s="13"/>
-      <c r="N14" s="13"/>
-      <c r="O14" s="13"/>
-      <c r="P14" s="13"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="12"/>
+      <c r="M14" s="12"/>
+      <c r="N14" s="12"/>
+      <c r="O14" s="12"/>
+      <c r="P14" s="12"/>
       <c r="Q14" s="13"/>
     </row>
     <row r="15" spans="1:17">
@@ -8118,19 +8199,19 @@
       <c r="C15" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
-      <c r="J15" s="13"/>
-      <c r="K15" s="13"/>
-      <c r="L15" s="13"/>
-      <c r="M15" s="13"/>
-      <c r="N15" s="13"/>
-      <c r="O15" s="13"/>
-      <c r="P15" s="13"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12"/>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="12"/>
+      <c r="P15" s="12"/>
       <c r="Q15" s="13"/>
     </row>
     <row r="16" spans="1:17">
@@ -8143,19 +8224,19 @@
       <c r="C16" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="13"/>
-      <c r="M16" s="13"/>
-      <c r="N16" s="13"/>
-      <c r="O16" s="13"/>
-      <c r="P16" s="13"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="12"/>
+      <c r="M16" s="12"/>
+      <c r="N16" s="12"/>
+      <c r="O16" s="12"/>
+      <c r="P16" s="12"/>
       <c r="Q16" s="13"/>
     </row>
     <row r="17" spans="1:17">
@@ -8168,78 +8249,77 @@
       <c r="C17" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="13"/>
-      <c r="N17" s="13"/>
-      <c r="O17" s="13"/>
-      <c r="P17" s="13"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="12"/>
+      <c r="P17" s="12"/>
       <c r="Q17" s="13"/>
     </row>
     <row r="20" spans="1:17">
       <c r="A20" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:17">
       <c r="A21" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="B21" s="13"/>
+        <v>76</v>
+      </c>
+      <c r="B21" s="12"/>
     </row>
     <row r="22" spans="1:17">
       <c r="A22" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="B22" s="13"/>
+        <v>77</v>
+      </c>
+      <c r="B22" s="12"/>
     </row>
     <row r="23" spans="1:17">
       <c r="A23" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="B23" s="13"/>
+        <v>78</v>
+      </c>
+      <c r="B23" s="12"/>
     </row>
     <row r="24" spans="1:17">
       <c r="A24" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="B24" s="13"/>
+        <v>79</v>
+      </c>
+      <c r="B24" s="12"/>
     </row>
     <row r="25" spans="1:17">
       <c r="A25" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="B25" s="13"/>
+        <v>80</v>
+      </c>
+      <c r="B25" s="12"/>
     </row>
     <row r="26" spans="1:17">
       <c r="A26" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="B26" s="13"/>
+        <v>81</v>
+      </c>
+      <c r="B26" s="12"/>
     </row>
     <row r="27" spans="1:17">
       <c r="A27" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="B27" s="13"/>
+        <v>82</v>
+      </c>
+      <c r="B27" s="12"/>
     </row>
     <row r="28" spans="1:17">
       <c r="A28" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="B28" s="13"/>
+        <v>83</v>
+      </c>
+      <c r="B28" s="12"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="A2:Q2"/>
   </mergeCells>
   <conditionalFormatting sqref="K6:K17">
     <cfRule type="colorScale" priority="1">
@@ -8267,22 +8347,635 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:R24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="13" width="11.7109375" customWidth="1"/>
+    <col min="14" max="17" width="13.7109375" customWidth="1"/>
+    <col min="18" max="18" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
+        <v>45351</v>
+      </c>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11"/>
+      <c r="O2" s="11"/>
+      <c r="P2" s="14"/>
+      <c r="Q2" s="14"/>
+      <c r="R2" s="11"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>45382</v>
+      </c>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="11"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="14"/>
+      <c r="Q3" s="14"/>
+      <c r="R3" s="11"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>45412</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="11"/>
+      <c r="M4" s="11"/>
+      <c r="N4" s="11"/>
+      <c r="O4" s="11"/>
+      <c r="P4" s="14"/>
+      <c r="Q4" s="14"/>
+      <c r="R4" s="11"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>45443</v>
+      </c>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+      <c r="N5" s="11"/>
+      <c r="O5" s="11"/>
+      <c r="P5" s="14"/>
+      <c r="Q5" s="14"/>
+      <c r="R5" s="11"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>45473</v>
+      </c>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+      <c r="N6" s="11"/>
+      <c r="O6" s="11"/>
+      <c r="P6" s="14"/>
+      <c r="Q6" s="14"/>
+      <c r="R6" s="11"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>45504</v>
+      </c>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
+      <c r="N7" s="11"/>
+      <c r="O7" s="11"/>
+      <c r="P7" s="14"/>
+      <c r="Q7" s="14"/>
+      <c r="R7" s="11"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
+        <v>45535</v>
+      </c>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="11"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11"/>
+      <c r="M8" s="11"/>
+      <c r="N8" s="11"/>
+      <c r="O8" s="11"/>
+      <c r="P8" s="14"/>
+      <c r="Q8" s="14"/>
+      <c r="R8" s="11"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
+        <v>45565</v>
+      </c>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="11"/>
+      <c r="N9" s="11"/>
+      <c r="O9" s="11"/>
+      <c r="P9" s="14"/>
+      <c r="Q9" s="14"/>
+      <c r="R9" s="11"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>45596</v>
+      </c>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="11"/>
+      <c r="N10" s="11"/>
+      <c r="O10" s="11"/>
+      <c r="P10" s="14"/>
+      <c r="Q10" s="14"/>
+      <c r="R10" s="11"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>45626</v>
+      </c>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="11"/>
+      <c r="M11" s="11"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="11"/>
+      <c r="P11" s="14"/>
+      <c r="Q11" s="14"/>
+      <c r="R11" s="11"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>45657</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="11"/>
+      <c r="N12" s="11"/>
+      <c r="O12" s="11"/>
+      <c r="P12" s="14"/>
+      <c r="Q12" s="14"/>
+      <c r="R12" s="11"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
+        <v>45688</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="11"/>
+      <c r="N13" s="11"/>
+      <c r="O13" s="11"/>
+      <c r="P13" s="14"/>
+      <c r="Q13" s="14"/>
+      <c r="R13" s="11"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>45716</v>
+      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="11"/>
+      <c r="O14" s="11"/>
+      <c r="P14" s="14"/>
+      <c r="Q14" s="14"/>
+      <c r="R14" s="11"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>45747</v>
+      </c>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="11"/>
+      <c r="N15" s="11"/>
+      <c r="O15" s="11"/>
+      <c r="P15" s="14"/>
+      <c r="Q15" s="14"/>
+      <c r="R15" s="11"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
+        <v>45777</v>
+      </c>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="11"/>
+      <c r="N16" s="11"/>
+      <c r="O16" s="11"/>
+      <c r="P16" s="14"/>
+      <c r="Q16" s="14"/>
+      <c r="R16" s="11"/>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>45808</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="11"/>
+      <c r="N17" s="11"/>
+      <c r="O17" s="11"/>
+      <c r="P17" s="14"/>
+      <c r="Q17" s="14"/>
+      <c r="R17" s="11"/>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
+        <v>45838</v>
+      </c>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="11"/>
+      <c r="M18" s="11"/>
+      <c r="N18" s="11"/>
+      <c r="O18" s="11"/>
+      <c r="P18" s="14"/>
+      <c r="Q18" s="14"/>
+      <c r="R18" s="11"/>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A19" s="3">
+        <v>45869</v>
+      </c>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="11"/>
+      <c r="M19" s="11"/>
+      <c r="N19" s="11"/>
+      <c r="O19" s="11"/>
+      <c r="P19" s="14"/>
+      <c r="Q19" s="14"/>
+      <c r="R19" s="11"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A20" s="3">
+        <v>45900</v>
+      </c>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="11"/>
+      <c r="M20" s="11"/>
+      <c r="N20" s="11"/>
+      <c r="O20" s="11"/>
+      <c r="P20" s="14"/>
+      <c r="Q20" s="14"/>
+      <c r="R20" s="11"/>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A21" s="3">
+        <v>45930</v>
+      </c>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="11"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="11"/>
+      <c r="M21" s="11"/>
+      <c r="N21" s="11"/>
+      <c r="O21" s="11"/>
+      <c r="P21" s="14"/>
+      <c r="Q21" s="14"/>
+      <c r="R21" s="11"/>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A22" s="3">
+        <v>45961</v>
+      </c>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="11"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="11"/>
+      <c r="M22" s="11"/>
+      <c r="N22" s="11"/>
+      <c r="O22" s="11"/>
+      <c r="P22" s="14"/>
+      <c r="Q22" s="14"/>
+      <c r="R22" s="11"/>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A23" s="3">
+        <v>45991</v>
+      </c>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="11"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="11"/>
+      <c r="M23" s="11"/>
+      <c r="N23" s="11"/>
+      <c r="O23" s="11"/>
+      <c r="P23" s="14"/>
+      <c r="Q23" s="14"/>
+      <c r="R23" s="11"/>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A24" s="3">
+        <v>46022</v>
+      </c>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
+      <c r="L24" s="11"/>
+      <c r="M24" s="11"/>
+      <c r="N24" s="11"/>
+      <c r="O24" s="11"/>
+      <c r="P24" s="14"/>
+      <c r="Q24" s="14"/>
+      <c r="R24" s="11"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="R2:R24">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFC00000"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{DA7ABA51-AAAA-BBBB-0004-000000000001}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{DA7ABA51-AAAA-BBBB-0004-000000000001}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFC00000"/>
+              <x14:negativeFillColor rgb="FFC00000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>R2:R24</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
-    <col min="2" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="7" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" customWidth="1"/>
+    <col min="4" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="7" width="14.7109375" customWidth="1"/>
     <col min="8" max="9" width="3.7109375" customWidth="1"/>
-    <col min="10" max="12" width="15.7109375" customWidth="1"/>
-    <col min="13" max="13" width="13.7109375" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" customWidth="1"/>
+    <col min="11" max="12" width="15.7109375" customWidth="1"/>
+    <col min="13" max="13" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8291,34 +8984,23 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-    </row>
     <row r="3" spans="1:13">
       <c r="J3" s="2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="K3" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="26" customHeight="1">
+      <c r="A4" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>2</v>
@@ -8330,19 +9012,19 @@
         <v>55</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="J4" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="K4" s="13"/>
-      <c r="L4" s="13"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
       <c r="M4" s="13"/>
     </row>
     <row r="5" spans="1:13">
@@ -8355,15 +9037,15 @@
       <c r="C5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
       <c r="J5" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="K5" s="13"/>
-      <c r="L5" s="13"/>
+      <c r="K5" s="12"/>
+      <c r="L5" s="12"/>
       <c r="M5" s="13"/>
     </row>
     <row r="6" spans="1:13">
@@ -8376,15 +9058,15 @@
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
       <c r="J6" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="12"/>
       <c r="M6" s="13"/>
     </row>
     <row r="7" spans="1:13">
@@ -8397,10 +9079,10 @@
       <c r="C7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="4" t="s">
@@ -8412,10 +9094,10 @@
       <c r="C8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="4" t="s">
@@ -8427,10 +9109,10 @@
       <c r="C9" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="4" t="s">
@@ -8442,10 +9124,10 @@
       <c r="C10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="4" t="s">
@@ -8457,10 +9139,10 @@
       <c r="C11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="4" t="s">
@@ -8472,10 +9154,10 @@
       <c r="C12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" s="4" t="s">
@@ -8487,10 +9169,10 @@
       <c r="C13" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="4" t="s">
@@ -8502,10 +9184,10 @@
       <c r="C14" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
     </row>
     <row r="15" spans="1:13">
       <c r="A15" s="4" t="s">
@@ -8517,10 +9199,10 @@
       <c r="C15" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="4" t="s">
@@ -8532,10 +9214,10 @@
       <c r="C16" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="4" t="s">
@@ -8547,10 +9229,10 @@
       <c r="C17" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="4" t="s">
@@ -8562,10 +9244,10 @@
       <c r="C18" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="4" t="s">
@@ -8577,10 +9259,10 @@
       <c r="C19" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="4" t="s">
@@ -8592,10 +9274,10 @@
       <c r="C20" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="4" t="s">
@@ -8607,10 +9289,10 @@
       <c r="C21" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
@@ -8622,10 +9304,10 @@
       <c r="C22" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
@@ -8637,10 +9319,10 @@
       <c r="C23" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
@@ -8652,10 +9334,10 @@
       <c r="C24" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
@@ -8667,10 +9349,10 @@
       <c r="C25" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" s="4" t="s">
@@ -8682,10 +9364,10 @@
       <c r="C26" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="13"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="4" t="s">
@@ -8697,10 +9379,10 @@
       <c r="C27" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="4" t="s">
@@ -8712,10 +9394,10 @@
       <c r="C28" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="13"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="12"/>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" s="4" t="s">
@@ -8727,10 +9409,10 @@
       <c r="C29" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="13"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" s="4" t="s">
@@ -8742,10 +9424,10 @@
       <c r="C30" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="4" t="s">
@@ -8757,10 +9439,10 @@
       <c r="C31" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="12"/>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" s="4" t="s">
@@ -8772,10 +9454,10 @@
       <c r="C32" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="12"/>
+      <c r="G32" s="12"/>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" s="4" t="s">
@@ -8787,10 +9469,10 @@
       <c r="C33" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="12"/>
+      <c r="G33" s="12"/>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" s="4" t="s">
@@ -8802,10 +9484,10 @@
       <c r="C34" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="13"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="12"/>
     </row>
     <row r="35" spans="1:7">
       <c r="A35" s="4" t="s">
@@ -8817,10 +9499,10 @@
       <c r="C35" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="12"/>
+      <c r="F35" s="12"/>
+      <c r="G35" s="12"/>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" s="4" t="s">
@@ -8832,10 +9514,10 @@
       <c r="C36" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="13"/>
-      <c r="G36" s="13"/>
+      <c r="D36" s="12"/>
+      <c r="E36" s="12"/>
+      <c r="F36" s="12"/>
+      <c r="G36" s="12"/>
     </row>
     <row r="37" spans="1:7">
       <c r="A37" s="4" t="s">
@@ -8847,10 +9529,10 @@
       <c r="C37" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="13"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
     </row>
     <row r="38" spans="1:7">
       <c r="A38" s="4" t="s">
@@ -8862,10 +9544,10 @@
       <c r="C38" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="13"/>
-      <c r="G38" s="13"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="4" t="s">
@@ -8877,10 +9559,10 @@
       <c r="C39" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="13"/>
+      <c r="D39" s="12"/>
+      <c r="E39" s="12"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="12"/>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" s="4" t="s">
@@ -8892,15 +9574,14 @@
       <c r="C40" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="13"/>
+      <c r="D40" s="12"/>
+      <c r="E40" s="12"/>
+      <c r="F40" s="12"/>
+      <c r="G40" s="12"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="G5:G40">
     <cfRule type="colorScale" priority="1">
@@ -8918,7 +9599,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8926,14 +9607,15 @@
     <col min="1" max="1" width="9.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" customWidth="1"/>
     <col min="3" max="3" width="14.7109375" customWidth="1"/>
-    <col min="4" max="5" width="15.7109375" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
     <col min="6" max="6" width="3.7109375" customWidth="1"/>
     <col min="7" max="12" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="28" customHeight="1">
+    <row r="1" spans="1:12" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8947,52 +9629,52 @@
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
     </row>
-    <row r="3" spans="1:12">
-      <c r="A3" s="14" t="s">
+    <row r="3" spans="1:12" ht="30" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="D3" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="D3" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="E3" s="14"/>
-      <c r="G3" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H3" s="14"/>
-      <c r="J3" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="K3" s="14"/>
+      <c r="E3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="H3" s="2"/>
+      <c r="J3" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="K3" s="2"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
+      <c r="A4" s="15"/>
+      <c r="B4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
     </row>
     <row r="5" spans="1:12">
-      <c r="A5" s="13"/>
-      <c r="B5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
+      <c r="A5" s="15"/>
+      <c r="B5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="30" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>2</v>
@@ -9004,7 +9686,7 @@
         <v>55</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -9012,45 +9694,45 @@
         <v>1</v>
       </c>
       <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="17"/>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="4">
         <v>2</v>
       </c>
       <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="17"/>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="4">
         <v>3</v>
       </c>
       <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="17"/>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="4">
         <v>4</v>
       </c>
       <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="17"/>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="4">
         <v>5</v>
       </c>
       <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -9066,4 +9748,906 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="8" width="14.7109375" customWidth="1"/>
+    <col min="9" max="11" width="16.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="3" spans="1:11" ht="26" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="3">
+        <v>45351</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="3">
+        <v>45382</v>
+      </c>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="3">
+        <v>45412</v>
+      </c>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="3">
+        <v>45443</v>
+      </c>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="3">
+        <v>45473</v>
+      </c>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="3">
+        <v>45504</v>
+      </c>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="3">
+        <v>45535</v>
+      </c>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="3">
+        <v>45565</v>
+      </c>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="3">
+        <v>45596</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="3">
+        <v>45626</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="3">
+        <v>45657</v>
+      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="3">
+        <v>45688</v>
+      </c>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" s="3">
+        <v>45716</v>
+      </c>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17" s="3">
+        <v>45747</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" s="3">
+        <v>45777</v>
+      </c>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19" s="3">
+        <v>45808</v>
+      </c>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" s="3">
+        <v>45838</v>
+      </c>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21" s="3">
+        <v>45869</v>
+      </c>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+    </row>
+    <row r="22" spans="1:11">
+      <c r="A22" s="3">
+        <v>45900</v>
+      </c>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+    </row>
+    <row r="23" spans="1:11">
+      <c r="A23" s="3">
+        <v>45930</v>
+      </c>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+    </row>
+    <row r="24" spans="1:11">
+      <c r="A24" s="3">
+        <v>45961</v>
+      </c>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+    </row>
+    <row r="25" spans="1:11">
+      <c r="A25" s="3">
+        <v>45991</v>
+      </c>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+    </row>
+    <row r="26" spans="1:11">
+      <c r="A26" s="3">
+        <v>46022</v>
+      </c>
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="11"/>
+    </row>
+    <row r="29" spans="1:11">
+      <c r="A29" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
+      <c r="A30" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
+    </row>
+    <row r="32" spans="1:11" ht="26" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11">
+      <c r="A33" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
+      <c r="I33" s="17"/>
+      <c r="J33" s="17"/>
+      <c r="K33" s="17"/>
+    </row>
+    <row r="34" spans="1:11">
+      <c r="A34" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+      <c r="I34" s="17"/>
+      <c r="J34" s="17"/>
+      <c r="K34" s="17"/>
+    </row>
+    <row r="35" spans="1:11">
+      <c r="A35" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B35" s="14"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="14"/>
+      <c r="I35" s="17"/>
+      <c r="J35" s="17"/>
+      <c r="K35" s="17"/>
+    </row>
+    <row r="36" spans="1:11">
+      <c r="A36" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B36" s="14"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="14"/>
+      <c r="I36" s="17"/>
+      <c r="J36" s="17"/>
+      <c r="K36" s="17"/>
+    </row>
+    <row r="37" spans="1:11">
+      <c r="A37" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="14"/>
+      <c r="H37" s="14"/>
+      <c r="I37" s="17"/>
+      <c r="J37" s="17"/>
+      <c r="K37" s="17"/>
+    </row>
+    <row r="38" spans="1:11">
+      <c r="A38" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14"/>
+      <c r="I38" s="17"/>
+      <c r="J38" s="17"/>
+      <c r="K38" s="17"/>
+    </row>
+    <row r="41" spans="1:11">
+      <c r="A41" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B41" s="14"/>
+    </row>
+    <row r="42" spans="1:11">
+      <c r="A42" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B42" s="17"/>
+    </row>
+    <row r="43" spans="1:11">
+      <c r="A43" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B43" s="17"/>
+    </row>
+    <row r="44" spans="1:11">
+      <c r="A44" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B44" s="17"/>
+    </row>
+    <row r="45" spans="1:11">
+      <c r="A45" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B45" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="I33:I38">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min" val="0"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O26"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="3" width="15.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="7" width="14.7109375" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="11" max="13" width="3.7109375" customWidth="1"/>
+    <col min="14" max="14" width="17.7109375" customWidth="1"/>
+    <col min="15" max="15" width="14.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15">
+      <c r="A1" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+    </row>
+    <row r="3" spans="1:15" ht="42" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="A4" s="3">
+        <v>45716</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="11"/>
+      <c r="N4" s="3">
+        <v>45351</v>
+      </c>
+      <c r="O4" s="11"/>
+    </row>
+    <row r="5" spans="1:15">
+      <c r="A5" s="3">
+        <v>45747</v>
+      </c>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="11"/>
+      <c r="N5" s="3">
+        <v>45382</v>
+      </c>
+      <c r="O5" s="11"/>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6" s="3">
+        <v>45777</v>
+      </c>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="11"/>
+      <c r="N6" s="3">
+        <v>45412</v>
+      </c>
+      <c r="O6" s="11"/>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7" s="3">
+        <v>45808</v>
+      </c>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="11"/>
+      <c r="N7" s="3">
+        <v>45443</v>
+      </c>
+      <c r="O7" s="11"/>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="A8" s="3">
+        <v>45838</v>
+      </c>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="11"/>
+      <c r="N8" s="3">
+        <v>45473</v>
+      </c>
+      <c r="O8" s="11"/>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" s="3">
+        <v>45869</v>
+      </c>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="11"/>
+      <c r="N9" s="3">
+        <v>45504</v>
+      </c>
+      <c r="O9" s="11"/>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="A10" s="3">
+        <v>45900</v>
+      </c>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="11"/>
+      <c r="N10" s="3">
+        <v>45535</v>
+      </c>
+      <c r="O10" s="11"/>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11" s="3">
+        <v>45930</v>
+      </c>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="11"/>
+      <c r="N11" s="3">
+        <v>45565</v>
+      </c>
+      <c r="O11" s="11"/>
+    </row>
+    <row r="12" spans="1:15">
+      <c r="A12" s="3">
+        <v>45961</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="14"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="11"/>
+      <c r="N12" s="3">
+        <v>45596</v>
+      </c>
+      <c r="O12" s="11"/>
+    </row>
+    <row r="13" spans="1:15">
+      <c r="A13" s="3">
+        <v>45991</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="11"/>
+      <c r="N13" s="3">
+        <v>45626</v>
+      </c>
+      <c r="O13" s="11"/>
+    </row>
+    <row r="14" spans="1:15">
+      <c r="A14" s="3">
+        <v>46022</v>
+      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="11"/>
+      <c r="N14" s="3">
+        <v>45657</v>
+      </c>
+      <c r="O14" s="11"/>
+    </row>
+    <row r="15" spans="1:15">
+      <c r="N15" s="3">
+        <v>45688</v>
+      </c>
+      <c r="O15" s="11"/>
+    </row>
+    <row r="16" spans="1:15">
+      <c r="N16" s="3">
+        <v>45716</v>
+      </c>
+      <c r="O16" s="11"/>
+    </row>
+    <row r="17" spans="1:15">
+      <c r="A17" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="B17" s="14"/>
+      <c r="N17" s="3">
+        <v>45747</v>
+      </c>
+      <c r="O17" s="11"/>
+    </row>
+    <row r="18" spans="1:15">
+      <c r="A18" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B18" s="11"/>
+      <c r="N18" s="3">
+        <v>45777</v>
+      </c>
+      <c r="O18" s="11"/>
+    </row>
+    <row r="19" spans="1:15">
+      <c r="A19" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="B19" s="14"/>
+      <c r="N19" s="3">
+        <v>45808</v>
+      </c>
+      <c r="O19" s="11"/>
+    </row>
+    <row r="20" spans="1:15">
+      <c r="A20" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B20" s="16"/>
+      <c r="N20" s="3">
+        <v>45838</v>
+      </c>
+      <c r="O20" s="11"/>
+    </row>
+    <row r="21" spans="1:15">
+      <c r="N21" s="3">
+        <v>45869</v>
+      </c>
+      <c r="O21" s="11"/>
+    </row>
+    <row r="22" spans="1:15">
+      <c r="N22" s="3">
+        <v>45900</v>
+      </c>
+      <c r="O22" s="11"/>
+    </row>
+    <row r="23" spans="1:15">
+      <c r="N23" s="3">
+        <v>45930</v>
+      </c>
+      <c r="O23" s="11"/>
+    </row>
+    <row r="24" spans="1:15">
+      <c r="N24" s="3">
+        <v>45961</v>
+      </c>
+      <c r="O24" s="11"/>
+    </row>
+    <row r="25" spans="1:15">
+      <c r="N25" s="3">
+        <v>45991</v>
+      </c>
+      <c r="O25" s="11"/>
+    </row>
+    <row r="26" spans="1:15">
+      <c r="N26" s="3">
+        <v>46022</v>
+      </c>
+      <c r="O26" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="H4:H14">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThanOrEqual">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Round 2 revision: remove all non-required background fills, unify fonts to single family/size
</commit_message>
<xml_diff>
--- a/股票组合风险分析_任务文件.xlsx
+++ b/股票组合风险分析_任务文件.xlsx
@@ -432,7 +432,7 @@
     <numFmt numFmtId="166" formatCode="¥#,##0;[Red]-¥#,##0"/>
     <numFmt numFmtId="167" formatCode="0.00%;[Red]-0.00%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -442,66 +442,19 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE7E6E6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEDEDED"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF5F5F5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF7E6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -531,10 +484,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -547,25 +500,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7746,7 +7689,7 @@
       <c r="D16" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="10">
         <f>SUM(E4:E15)</f>
         <v>1.0</v>
       </c>
@@ -7974,20 +7917,20 @@
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12"/>
-      <c r="N6" s="12"/>
-      <c r="O6" s="12"/>
-      <c r="P6" s="12"/>
-      <c r="Q6" s="13"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="4"/>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" s="4" t="s">
@@ -7999,20 +7942,20 @@
       <c r="C7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
-      <c r="M7" s="12"/>
-      <c r="N7" s="12"/>
-      <c r="O7" s="12"/>
-      <c r="P7" s="12"/>
-      <c r="Q7" s="13"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="4"/>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" s="4" t="s">
@@ -8024,20 +7967,20 @@
       <c r="C8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="12"/>
-      <c r="P8" s="12"/>
-      <c r="Q8" s="13"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="4"/>
     </row>
     <row r="9" spans="1:17">
       <c r="A9" s="4" t="s">
@@ -8049,20 +7992,20 @@
       <c r="C9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
-      <c r="M9" s="12"/>
-      <c r="N9" s="12"/>
-      <c r="O9" s="12"/>
-      <c r="P9" s="12"/>
-      <c r="Q9" s="13"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="4"/>
     </row>
     <row r="10" spans="1:17">
       <c r="A10" s="4" t="s">
@@ -8074,20 +8017,20 @@
       <c r="C10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="12"/>
-      <c r="M10" s="12"/>
-      <c r="N10" s="12"/>
-      <c r="O10" s="12"/>
-      <c r="P10" s="12"/>
-      <c r="Q10" s="13"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="4"/>
     </row>
     <row r="11" spans="1:17">
       <c r="A11" s="4" t="s">
@@ -8099,20 +8042,20 @@
       <c r="C11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="12"/>
-      <c r="M11" s="12"/>
-      <c r="N11" s="12"/>
-      <c r="O11" s="12"/>
-      <c r="P11" s="12"/>
-      <c r="Q11" s="13"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="4"/>
     </row>
     <row r="12" spans="1:17">
       <c r="A12" s="4" t="s">
@@ -8124,20 +8067,20 @@
       <c r="C12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="12"/>
-      <c r="M12" s="12"/>
-      <c r="N12" s="12"/>
-      <c r="O12" s="12"/>
-      <c r="P12" s="12"/>
-      <c r="Q12" s="13"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="4"/>
     </row>
     <row r="13" spans="1:17">
       <c r="A13" s="4" t="s">
@@ -8149,20 +8092,20 @@
       <c r="C13" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="12"/>
-      <c r="N13" s="12"/>
-      <c r="O13" s="12"/>
-      <c r="P13" s="12"/>
-      <c r="Q13" s="13"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="4"/>
     </row>
     <row r="14" spans="1:17">
       <c r="A14" s="4" t="s">
@@ -8174,20 +8117,20 @@
       <c r="C14" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="12"/>
-      <c r="M14" s="12"/>
-      <c r="N14" s="12"/>
-      <c r="O14" s="12"/>
-      <c r="P14" s="12"/>
-      <c r="Q14" s="13"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
+      <c r="Q14" s="4"/>
     </row>
     <row r="15" spans="1:17">
       <c r="A15" s="4" t="s">
@@ -8199,20 +8142,20 @@
       <c r="C15" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
-      <c r="L15" s="12"/>
-      <c r="M15" s="12"/>
-      <c r="N15" s="12"/>
-      <c r="O15" s="12"/>
-      <c r="P15" s="12"/>
-      <c r="Q15" s="13"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="4"/>
     </row>
     <row r="16" spans="1:17">
       <c r="A16" s="4" t="s">
@@ -8224,20 +8167,20 @@
       <c r="C16" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="12"/>
-      <c r="L16" s="12"/>
-      <c r="M16" s="12"/>
-      <c r="N16" s="12"/>
-      <c r="O16" s="12"/>
-      <c r="P16" s="12"/>
-      <c r="Q16" s="13"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
+      <c r="O16" s="8"/>
+      <c r="P16" s="8"/>
+      <c r="Q16" s="4"/>
     </row>
     <row r="17" spans="1:17">
       <c r="A17" s="4" t="s">
@@ -8249,20 +8192,20 @@
       <c r="C17" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="12"/>
-      <c r="L17" s="12"/>
-      <c r="M17" s="12"/>
-      <c r="N17" s="12"/>
-      <c r="O17" s="12"/>
-      <c r="P17" s="12"/>
-      <c r="Q17" s="13"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="8"/>
+      <c r="N17" s="8"/>
+      <c r="O17" s="8"/>
+      <c r="P17" s="8"/>
+      <c r="Q17" s="4"/>
     </row>
     <row r="20" spans="1:17">
       <c r="A20" s="7" t="s">
@@ -8273,49 +8216,49 @@
       <c r="A21" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B21" s="12"/>
+      <c r="B21" s="8"/>
     </row>
     <row r="22" spans="1:17">
       <c r="A22" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="B22" s="12"/>
+      <c r="B22" s="8"/>
     </row>
     <row r="23" spans="1:17">
       <c r="A23" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B23" s="12"/>
+      <c r="B23" s="8"/>
     </row>
     <row r="24" spans="1:17">
       <c r="A24" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B24" s="12"/>
+      <c r="B24" s="8"/>
     </row>
     <row r="25" spans="1:17">
       <c r="A25" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B25" s="12"/>
+      <c r="B25" s="8"/>
     </row>
     <row r="26" spans="1:17">
       <c r="A26" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B26" s="12"/>
+      <c r="B26" s="8"/>
     </row>
     <row r="27" spans="1:17">
       <c r="A27" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B27" s="12"/>
+      <c r="B27" s="8"/>
     </row>
     <row r="28" spans="1:17">
       <c r="A28" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B28" s="12"/>
+      <c r="B28" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -8417,507 +8360,507 @@
       <c r="A2" s="3">
         <v>45351</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="14"/>
-      <c r="Q2" s="14"/>
-      <c r="R2" s="11"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="10"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>45382</v>
       </c>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="11"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="10"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>45412</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="14"/>
-      <c r="Q4" s="14"/>
-      <c r="R4" s="11"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="10"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>45443</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
-      <c r="O5" s="11"/>
-      <c r="P5" s="14"/>
-      <c r="Q5" s="14"/>
-      <c r="R5" s="11"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="10"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>45473</v>
       </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="14"/>
-      <c r="Q6" s="14"/>
-      <c r="R6" s="11"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="10"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>45504</v>
       </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="14"/>
-      <c r="Q7" s="14"/>
-      <c r="R7" s="11"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="10"/>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>45535</v>
       </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="11"/>
-      <c r="O8" s="11"/>
-      <c r="P8" s="14"/>
-      <c r="Q8" s="14"/>
-      <c r="R8" s="11"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="6"/>
+      <c r="Q8" s="6"/>
+      <c r="R8" s="10"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>45565</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
-      <c r="O9" s="11"/>
-      <c r="P9" s="14"/>
-      <c r="Q9" s="14"/>
-      <c r="R9" s="11"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+      <c r="P9" s="6"/>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="10"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>45596</v>
       </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="11"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="11"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="11"/>
-      <c r="O10" s="11"/>
-      <c r="P10" s="14"/>
-      <c r="Q10" s="14"/>
-      <c r="R10" s="11"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
+      <c r="P10" s="6"/>
+      <c r="Q10" s="6"/>
+      <c r="R10" s="10"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>45626</v>
       </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="11"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="14"/>
-      <c r="Q11" s="14"/>
-      <c r="R11" s="11"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="6"/>
+      <c r="Q11" s="6"/>
+      <c r="R11" s="10"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>45657</v>
       </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="11"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="14"/>
-      <c r="Q12" s="14"/>
-      <c r="R12" s="11"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="6"/>
+      <c r="R12" s="10"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>45688</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="11"/>
-      <c r="P13" s="14"/>
-      <c r="Q13" s="14"/>
-      <c r="R13" s="11"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="10"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="10"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>45716</v>
       </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="11"/>
-      <c r="O14" s="11"/>
-      <c r="P14" s="14"/>
-      <c r="Q14" s="14"/>
-      <c r="R14" s="11"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="10"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="6"/>
+      <c r="R14" s="10"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>45747</v>
       </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="11"/>
-      <c r="P15" s="14"/>
-      <c r="Q15" s="14"/>
-      <c r="R15" s="11"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+      <c r="P15" s="6"/>
+      <c r="Q15" s="6"/>
+      <c r="R15" s="10"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>45777</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
-      <c r="O16" s="11"/>
-      <c r="P16" s="14"/>
-      <c r="Q16" s="14"/>
-      <c r="R16" s="11"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+      <c r="O16" s="10"/>
+      <c r="P16" s="6"/>
+      <c r="Q16" s="6"/>
+      <c r="R16" s="10"/>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>45808</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11"/>
-      <c r="O17" s="11"/>
-      <c r="P17" s="14"/>
-      <c r="Q17" s="14"/>
-      <c r="R17" s="11"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
+      <c r="P17" s="6"/>
+      <c r="Q17" s="6"/>
+      <c r="R17" s="10"/>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>45838</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
-      <c r="O18" s="11"/>
-      <c r="P18" s="14"/>
-      <c r="Q18" s="14"/>
-      <c r="R18" s="11"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+      <c r="P18" s="6"/>
+      <c r="Q18" s="6"/>
+      <c r="R18" s="10"/>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>45869</v>
       </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11"/>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11"/>
-      <c r="O19" s="11"/>
-      <c r="P19" s="14"/>
-      <c r="Q19" s="14"/>
-      <c r="R19" s="11"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+      <c r="P19" s="6"/>
+      <c r="Q19" s="6"/>
+      <c r="R19" s="10"/>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>45900</v>
       </c>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11"/>
-      <c r="L20" s="11"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11"/>
-      <c r="O20" s="11"/>
-      <c r="P20" s="14"/>
-      <c r="Q20" s="14"/>
-      <c r="R20" s="11"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="6"/>
+      <c r="Q20" s="6"/>
+      <c r="R20" s="10"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>45930</v>
       </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
-      <c r="O21" s="11"/>
-      <c r="P21" s="14"/>
-      <c r="Q21" s="14"/>
-      <c r="R21" s="11"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
+      <c r="P21" s="6"/>
+      <c r="Q21" s="6"/>
+      <c r="R21" s="10"/>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>45961</v>
       </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
-      <c r="O22" s="11"/>
-      <c r="P22" s="14"/>
-      <c r="Q22" s="14"/>
-      <c r="R22" s="11"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10"/>
+      <c r="O22" s="10"/>
+      <c r="P22" s="6"/>
+      <c r="Q22" s="6"/>
+      <c r="R22" s="10"/>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>45991</v>
       </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="11"/>
-      <c r="L23" s="11"/>
-      <c r="M23" s="11"/>
-      <c r="N23" s="11"/>
-      <c r="O23" s="11"/>
-      <c r="P23" s="14"/>
-      <c r="Q23" s="14"/>
-      <c r="R23" s="11"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="6"/>
+      <c r="Q23" s="6"/>
+      <c r="R23" s="10"/>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>46022</v>
       </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11"/>
-      <c r="L24" s="11"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
-      <c r="O24" s="11"/>
-      <c r="P24" s="14"/>
-      <c r="Q24" s="14"/>
-      <c r="R24" s="11"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="10"/>
+      <c r="O24" s="10"/>
+      <c r="P24" s="6"/>
+      <c r="Q24" s="6"/>
+      <c r="R24" s="10"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="R2:R24">
@@ -9023,9 +8966,9 @@
       <c r="J4" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="K4" s="12"/>
-      <c r="L4" s="12"/>
-      <c r="M4" s="13"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="4"/>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="4" t="s">
@@ -9037,16 +8980,16 @@
       <c r="C5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
       <c r="J5" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="13"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="4"/>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="4" t="s">
@@ -9058,16 +9001,16 @@
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
       <c r="J6" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="13"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="4"/>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="4" t="s">
@@ -9079,10 +9022,10 @@
       <c r="C7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="4" t="s">
@@ -9094,10 +9037,10 @@
       <c r="C8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="4" t="s">
@@ -9109,10 +9052,10 @@
       <c r="C9" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="4" t="s">
@@ -9124,10 +9067,10 @@
       <c r="C10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="4" t="s">
@@ -9139,10 +9082,10 @@
       <c r="C11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="4" t="s">
@@ -9154,10 +9097,10 @@
       <c r="C12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" s="4" t="s">
@@ -9169,10 +9112,10 @@
       <c r="C13" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="4" t="s">
@@ -9184,10 +9127,10 @@
       <c r="C14" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
     </row>
     <row r="15" spans="1:13">
       <c r="A15" s="4" t="s">
@@ -9199,10 +9142,10 @@
       <c r="C15" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="4" t="s">
@@ -9214,10 +9157,10 @@
       <c r="C16" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="4" t="s">
@@ -9229,10 +9172,10 @@
       <c r="C17" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="4" t="s">
@@ -9244,10 +9187,10 @@
       <c r="C18" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="4" t="s">
@@ -9259,10 +9202,10 @@
       <c r="C19" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="4" t="s">
@@ -9274,10 +9217,10 @@
       <c r="C20" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="4" t="s">
@@ -9289,10 +9232,10 @@
       <c r="C21" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
@@ -9304,10 +9247,10 @@
       <c r="C22" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
@@ -9319,10 +9262,10 @@
       <c r="C23" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
@@ -9334,10 +9277,10 @@
       <c r="C24" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-      <c r="G24" s="12"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
@@ -9349,10 +9292,10 @@
       <c r="C25" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" s="4" t="s">
@@ -9364,10 +9307,10 @@
       <c r="C26" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="4" t="s">
@@ -9379,10 +9322,10 @@
       <c r="C27" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="4" t="s">
@@ -9394,10 +9337,10 @@
       <c r="C28" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="12"/>
-      <c r="G28" s="12"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" s="4" t="s">
@@ -9409,10 +9352,10 @@
       <c r="C29" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" s="4" t="s">
@@ -9424,10 +9367,10 @@
       <c r="C30" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
-      <c r="G30" s="12"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="4" t="s">
@@ -9439,10 +9382,10 @@
       <c r="C31" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" s="4" t="s">
@@ -9454,10 +9397,10 @@
       <c r="C32" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="12"/>
-      <c r="G32" s="12"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" s="4" t="s">
@@ -9469,10 +9412,10 @@
       <c r="C33" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" s="4" t="s">
@@ -9484,10 +9427,10 @@
       <c r="C34" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D34" s="12"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
-      <c r="G34" s="12"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
     </row>
     <row r="35" spans="1:7">
       <c r="A35" s="4" t="s">
@@ -9499,10 +9442,10 @@
       <c r="C35" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D35" s="12"/>
-      <c r="E35" s="12"/>
-      <c r="F35" s="12"/>
-      <c r="G35" s="12"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" s="4" t="s">
@@ -9514,10 +9457,10 @@
       <c r="C36" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
-      <c r="G36" s="12"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
     </row>
     <row r="37" spans="1:7">
       <c r="A37" s="4" t="s">
@@ -9529,10 +9472,10 @@
       <c r="C37" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D37" s="12"/>
-      <c r="E37" s="12"/>
-      <c r="F37" s="12"/>
-      <c r="G37" s="12"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
     </row>
     <row r="38" spans="1:7">
       <c r="A38" s="4" t="s">
@@ -9544,10 +9487,10 @@
       <c r="C38" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
-      <c r="F38" s="12"/>
-      <c r="G38" s="12"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="4" t="s">
@@ -9559,10 +9502,10 @@
       <c r="C39" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D39" s="12"/>
-      <c r="E39" s="12"/>
-      <c r="F39" s="12"/>
-      <c r="G39" s="12"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" s="4" t="s">
@@ -9574,10 +9517,10 @@
       <c r="C40" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D40" s="12"/>
-      <c r="E40" s="12"/>
-      <c r="F40" s="12"/>
-      <c r="G40" s="12"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -9648,24 +9591,24 @@
       <c r="K3" s="2"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="15"/>
-      <c r="B4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11"/>
     </row>
     <row r="5" spans="1:12">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="7" t="s">
@@ -9693,46 +9636,46 @@
       <c r="A9" s="4">
         <v>1</v>
       </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="17"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="9"/>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="4">
         <v>2</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="17"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="9"/>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="4">
         <v>3</v>
       </c>
-      <c r="B11" s="13"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="17"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="9"/>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="4">
         <v>4</v>
       </c>
-      <c r="B12" s="13"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="17"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="9"/>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="4">
         <v>5</v>
       </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="17"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -9805,277 +9748,277 @@
       <c r="A4" s="3">
         <v>45351</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="3">
         <v>45382</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="3">
         <v>45412</v>
       </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="3">
         <v>45443</v>
       </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="3">
         <v>45473</v>
       </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="3">
         <v>45504</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="3">
         <v>45535</v>
       </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="3">
         <v>45565</v>
       </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="3">
         <v>45596</v>
       </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="3">
         <v>45626</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="3">
         <v>45657</v>
       </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="3">
         <v>45688</v>
       </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="3">
         <v>45716</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="3">
         <v>45747</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="3">
         <v>45777</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="3">
         <v>45808</v>
       </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="3">
         <v>45838</v>
       </c>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="3">
         <v>45869</v>
       </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="3">
         <v>45900</v>
       </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="3">
         <v>45930</v>
       </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="3">
         <v>45961</v>
       </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="3">
         <v>45991</v>
       </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="3">
         <v>46022</v>
       </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" s="2" t="s">
@@ -10104,12 +10047,12 @@
       <c r="A30" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="11"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
     </row>
     <row r="32" spans="1:11" ht="26" customHeight="1">
       <c r="A32" s="2" t="s">
@@ -10150,121 +10093,121 @@
       <c r="A33" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="17"/>
-      <c r="K33" s="17"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
     </row>
     <row r="34" spans="1:11">
       <c r="A34" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="17"/>
-      <c r="J34" s="17"/>
-      <c r="K34" s="17"/>
+      <c r="B34" s="6"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
     </row>
     <row r="35" spans="1:11">
       <c r="A35" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="17"/>
-      <c r="J35" s="17"/>
-      <c r="K35" s="17"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
     </row>
     <row r="36" spans="1:11">
       <c r="A36" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="17"/>
-      <c r="J36" s="17"/>
-      <c r="K36" s="17"/>
+      <c r="B36" s="6"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
     </row>
     <row r="37" spans="1:11">
       <c r="A37" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="17"/>
-      <c r="J37" s="17"/>
-      <c r="K37" s="17"/>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="9"/>
+      <c r="J37" s="9"/>
+      <c r="K37" s="9"/>
     </row>
     <row r="38" spans="1:11">
       <c r="A38" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="17"/>
-      <c r="J38" s="17"/>
-      <c r="K38" s="17"/>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+      <c r="I38" s="9"/>
+      <c r="J38" s="9"/>
+      <c r="K38" s="9"/>
     </row>
     <row r="41" spans="1:11">
       <c r="A41" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="B41" s="14"/>
+      <c r="B41" s="6"/>
     </row>
     <row r="42" spans="1:11">
       <c r="A42" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B42" s="17"/>
+      <c r="B42" s="9"/>
     </row>
     <row r="43" spans="1:11">
       <c r="A43" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="B43" s="17"/>
+      <c r="B43" s="9"/>
     </row>
     <row r="44" spans="1:11">
       <c r="A44" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="B44" s="17"/>
+      <c r="B44" s="9"/>
     </row>
     <row r="45" spans="1:11">
       <c r="A45" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="B45" s="16"/>
+      <c r="B45" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -10357,287 +10300,287 @@
       <c r="A4" s="3">
         <v>45716</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="11"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="10"/>
       <c r="N4" s="3">
         <v>45351</v>
       </c>
-      <c r="O4" s="11"/>
+      <c r="O4" s="10"/>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="3">
         <v>45747</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="11"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="10"/>
       <c r="N5" s="3">
         <v>45382</v>
       </c>
-      <c r="O5" s="11"/>
+      <c r="O5" s="10"/>
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="3">
         <v>45777</v>
       </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="11"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="10"/>
       <c r="N6" s="3">
         <v>45412</v>
       </c>
-      <c r="O6" s="11"/>
+      <c r="O6" s="10"/>
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="3">
         <v>45808</v>
       </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="11"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="10"/>
       <c r="N7" s="3">
         <v>45443</v>
       </c>
-      <c r="O7" s="11"/>
+      <c r="O7" s="10"/>
     </row>
     <row r="8" spans="1:15">
       <c r="A8" s="3">
         <v>45838</v>
       </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="11"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="10"/>
       <c r="N8" s="3">
         <v>45473</v>
       </c>
-      <c r="O8" s="11"/>
+      <c r="O8" s="10"/>
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="3">
         <v>45869</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
-      <c r="J9" s="11"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="10"/>
       <c r="N9" s="3">
         <v>45504</v>
       </c>
-      <c r="O9" s="11"/>
+      <c r="O9" s="10"/>
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="3">
         <v>45900</v>
       </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="11"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="10"/>
       <c r="N10" s="3">
         <v>45535</v>
       </c>
-      <c r="O10" s="11"/>
+      <c r="O10" s="10"/>
     </row>
     <row r="11" spans="1:15">
       <c r="A11" s="3">
         <v>45930</v>
       </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="11"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="10"/>
       <c r="N11" s="3">
         <v>45565</v>
       </c>
-      <c r="O11" s="11"/>
+      <c r="O11" s="10"/>
     </row>
     <row r="12" spans="1:15">
       <c r="A12" s="3">
         <v>45961</v>
       </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="11"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="10"/>
       <c r="N12" s="3">
         <v>45596</v>
       </c>
-      <c r="O12" s="11"/>
+      <c r="O12" s="10"/>
     </row>
     <row r="13" spans="1:15">
       <c r="A13" s="3">
         <v>45991</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="11"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="10"/>
       <c r="N13" s="3">
         <v>45626</v>
       </c>
-      <c r="O13" s="11"/>
+      <c r="O13" s="10"/>
     </row>
     <row r="14" spans="1:15">
       <c r="A14" s="3">
         <v>46022</v>
       </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
-      <c r="J14" s="11"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="10"/>
       <c r="N14" s="3">
         <v>45657</v>
       </c>
-      <c r="O14" s="11"/>
+      <c r="O14" s="10"/>
     </row>
     <row r="15" spans="1:15">
       <c r="N15" s="3">
         <v>45688</v>
       </c>
-      <c r="O15" s="11"/>
+      <c r="O15" s="10"/>
     </row>
     <row r="16" spans="1:15">
       <c r="N16" s="3">
         <v>45716</v>
       </c>
-      <c r="O16" s="11"/>
+      <c r="O16" s="10"/>
     </row>
     <row r="17" spans="1:15">
       <c r="A17" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="B17" s="14"/>
+      <c r="B17" s="6"/>
       <c r="N17" s="3">
         <v>45747</v>
       </c>
-      <c r="O17" s="11"/>
+      <c r="O17" s="10"/>
     </row>
     <row r="18" spans="1:15">
       <c r="A18" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="B18" s="11"/>
+      <c r="B18" s="10"/>
       <c r="N18" s="3">
         <v>45777</v>
       </c>
-      <c r="O18" s="11"/>
+      <c r="O18" s="10"/>
     </row>
     <row r="19" spans="1:15">
       <c r="A19" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B19" s="14"/>
+      <c r="B19" s="6"/>
       <c r="N19" s="3">
         <v>45808</v>
       </c>
-      <c r="O19" s="11"/>
+      <c r="O19" s="10"/>
     </row>
     <row r="20" spans="1:15">
       <c r="A20" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="B20" s="16"/>
+      <c r="B20" s="5"/>
       <c r="N20" s="3">
         <v>45838</v>
       </c>
-      <c r="O20" s="11"/>
+      <c r="O20" s="10"/>
     </row>
     <row r="21" spans="1:15">
       <c r="N21" s="3">
         <v>45869</v>
       </c>
-      <c r="O21" s="11"/>
+      <c r="O21" s="10"/>
     </row>
     <row r="22" spans="1:15">
       <c r="N22" s="3">
         <v>45900</v>
       </c>
-      <c r="O22" s="11"/>
+      <c r="O22" s="10"/>
     </row>
     <row r="23" spans="1:15">
       <c r="N23" s="3">
         <v>45930</v>
       </c>
-      <c r="O23" s="11"/>
+      <c r="O23" s="10"/>
     </row>
     <row r="24" spans="1:15">
       <c r="N24" s="3">
         <v>45961</v>
       </c>
-      <c r="O24" s="11"/>
+      <c r="O24" s="10"/>
     </row>
     <row r="25" spans="1:15">
       <c r="N25" s="3">
         <v>45991</v>
       </c>
-      <c r="O25" s="11"/>
+      <c r="O25" s="10"/>
     </row>
     <row r="26" spans="1:15">
       <c r="N26" s="3">
         <v>46022</v>
       </c>
-      <c r="O26" s="11"/>
+      <c r="O26" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>